<commit_message>
pip2 forces added - no bugs - 1250 frames
</commit_message>
<xml_diff>
--- a/results_G2/ch2_permation_residue_comb.xlsx
+++ b/results_G2/ch2_permation_residue_comb.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,7 +513,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>130, 130, 426, 786</t>
+          <t>130, 426</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -573,20 +573,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>98, 130, 786, SF</t>
+          <t>130, 786</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>786</t>
+          <t>786, 130</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>959, 1219</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>98, 130, 786, 1082</t>
+          <t>98, 786, 1082</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -633,7 +633,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>98, 426, 1082, SF, SF</t>
+          <t>98, 1082, SF</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -653,7 +653,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>98, 458, 754, 786, 1082</t>
+          <t>754, 786, 1082</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -673,7 +673,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>98, 458, 754, 1082</t>
+          <t>458</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -693,7 +693,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>130, 426, 786, SF, SF</t>
+          <t>786</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -707,26 +707,6 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>1225</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>98, 130, 754, 786, 1082, SF</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>1219</t>
         </is>
       </c>
     </row>

</xml_diff>